<commit_message>
fix(pizza-shop-en): revisión final aplicada (4 B · 6 M · 23 m) — G1-G9 VERDE, regresión 27/27
B1 tarjeta duplicada en el hub EN · B2 tarea de la beer & wine license · B3/M1 gas y VPN coherentes con la AVPN ·
B4 cuota de plataforma 12 % + guarda «10 % of sales» · M4/M5 textos ajustados a la calculadora · M6 extintores.
Detalle en business-plans-en-8/REVISION-FINAL.md §5.

Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/pizza-shop-business-plan/pizza-shop-financial-projections.xlsx
+++ b/astro-site/public/dl/pizza-shop-business-plan/pizza-shop-financial-projections.xlsx
@@ -751,7 +751,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Equivalent covers per day, year-1 average: about 47 dine-in (patio included from April through October) and about 15 from take-out and delivery, which are the orders (about 10 a day at about $52 excl. sales tax: 2 pizzas, a starter and a drink) divided by the average check. A Saturday runs about 110; a Tuesday, about 45 (Kit estimate). Compare it with the foot traffic on your street on a Friday night and a Tuesday at lunch</t>
+          <t>Equivalent covers per day, year-1 average: about 47 dine-in (patio included from April through October) and about 15 from take-out and delivery, which are the orders (about 10 a day at about $54 excl. sales tax: 2 pizzas, a starter and a drink) divided by the average check. A Saturday runs about 110; a Tuesday, about 45 (Kit estimate). Compare it with the foot traffic on your street on a Friday night and a Tuesday at lunch</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>365 days minus 52 closed Mondays, the main holidays (Thanksgiving, Christmas, New Year's Day, July 4) and a week in January for oven maintenance and vacation, rounded to 300. It is the SAME figure for the P&amp;L, break-even, scenarios and staffing hours</t>
+          <t>365 days minus 52 closed Mondays, the main holidays (Thanksgiving, Christmas, New Year's Day, July 4) and two weeks in January for oven maintenance and vacation, rounded to 300. It is the SAME figure for the P&amp;L, break-even, scenarios and staffing hours</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>General liability, liquor liability (beer &amp; wine), property coverage that names the open-flame oven, and workers' comp. Tell the carrier the oven is wood-fired: it changes the premium and the terms. Rates vary by state, so get at least two quotes</t>
+          <t>General liability, liquor liability (beer &amp; wine) and property coverage that names the open-flame oven (workers' comp is in the payroll tax rate above). Tell the carrier the oven is wood-fired: it changes the premium and the terms. Rates vary by state, so get at least two quotes</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>For about six pizzas at a time, UL 2162-listed. Forno Bravo posts $12,950 for its Modena120 (48 in); Marra Forni, Acunto and Ferrara publish no price. The range is $12,950-$25,000+ (Oct 2026); ask for a quote that includes installation. A gas or electric oven is a variant and does not qualify for VPN certification</t>
+          <t>For about six pizzas at a time, UL 2162-listed. Forno Bravo posts $12,950 for its Modena120 (48 in); Marra Forni, Acunto and Ferrara publish no price. The range is $12,950-$25,000+ (Oct 2026); ask for a quote that includes installation. A gas or electric oven is a variant: an electric oven never qualifies for VPN certification, and a gas oven only where wood burning is forbidden and documented</t>
         </is>
       </c>
       <c r="E12" s="32" t="inlineStr">
@@ -6196,7 +6196,7 @@
       <c r="I20" s="29" t="n"/>
       <c r="J20" s="29" t="inlineStr">
         <is>
-          <t>50 weeks: 52 minus about two weeks of vacation, holidays and average absences. There is no federal vacation requirement in the US: adjust it to your own policy</t>
+          <t>46 weeks: 52 minus about six weeks for vacation, holidays, the January closure and average absences. There is no federal vacation requirement in the US: adjust it to your own policy</t>
         </is>
       </c>
     </row>
@@ -6975,7 +6975,7 @@
       </c>
       <c r="B38" s="29" t="inlineStr">
         <is>
-          <t>1 quart (1 liter) of water per ~4 lb (1.8 kg) of flour, 50-55 g of salt, 3 g of fresh yeast</t>
+          <t>1.06 quarts (1 liter) of water per ~4 lb (1.8 kg) of flour, 50-55 g of salt, 3 g of fresh yeast</t>
         </is>
       </c>
       <c r="C38" s="29" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="D39" s="48" t="inlineStr">
         <is>
-          <t>Wood-fired dome oven; gas or electric is a variant and does not qualify for VPN</t>
+          <t>Wood-fired dome oven; gas only where wood is banned (documented); electric does not qualify for VPN</t>
         </is>
       </c>
       <c r="E39" s="29" t="n"/>
@@ -7031,7 +7031,7 @@
       </c>
       <c r="D40" s="48" t="inlineStr">
         <is>
-          <t>$2,500 certification + $300 inspection + $400 a year (USA/Canada); needs an open location and a wood-fired dome oven</t>
+          <t>$2,500 certification + $300 inspection + $400 a year (USA/Canada); needs an open location and a wood-fired dome oven (gas only where wood is banned)</t>
         </is>
       </c>
       <c r="E40" s="29" t="n"/>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="O20" s="29" t="inlineStr">
         <is>
-          <t>Cash only leaves when the quarter's result is positive. Months without a settlement are left blank, not zero. The cell turns RED when the payment takes more cash than is left that month. The model settles quarterly (April, July, October, January): if your state requires monthly filing, expect smaller payments every month instead</t>
+          <t>Cash only leaves when the quarter's result is positive. Months without a settlement are left blank, not zero. The cell turns RED when the payment takes more cash than is left that month. The model settles quarterly, in the month after each plan quarter (Months 4, 7 and 10: December, March and June with Month 1 in September; the fourth quarter is remitted in Month 13): if your state requires monthly filing, expect smaller payments every month instead</t>
         </is>
       </c>
     </row>

</xml_diff>